<commit_message>
Creacion de archivos scv
</commit_message>
<xml_diff>
--- a/data/DATA_inicial.xlsx
+++ b/data/DATA_inicial.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\72358\Desktop\DB[1]\Carpeta Práctica 2-20260302\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49BA2D8A-8C9C-4672-9956-21EDED9B9F55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1006A1D-0598-4E46-B026-5B8E3BDBAF89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="4500" windowWidth="20730" windowHeight="11040" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20610" yWindow="4500" windowWidth="20730" windowHeight="11040" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESPUESTA_USUARIO" sheetId="7" r:id="rId1"/>
@@ -1588,15 +1588,27 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1611,11 +1623,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1649,6 +1676,18 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8267,71 +8306,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="13" t="s">
         <v>375</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="13" t="s">
         <v>376</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="13" t="s">
         <v>377</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="13" t="s">
         <v>378</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="13" t="s">
         <v>379</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="15" t="s">
         <v>380</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="15" t="s">
         <v>381</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2">
-        <v>1</v>
-      </c>
-      <c r="E2" s="2">
-        <v>1</v>
-      </c>
-      <c r="F2" s="2">
-        <v>1</v>
-      </c>
-      <c r="G2" s="2">
+      <c r="A2" s="14">
+        <v>1</v>
+      </c>
+      <c r="B2" s="14">
+        <v>1</v>
+      </c>
+      <c r="C2" s="14">
+        <v>1</v>
+      </c>
+      <c r="D2" s="14">
+        <v>1</v>
+      </c>
+      <c r="E2" s="14">
+        <v>1</v>
+      </c>
+      <c r="F2" s="16">
+        <v>1</v>
+      </c>
+      <c r="G2" s="16">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2">
-        <v>2</v>
-      </c>
-      <c r="C3" s="2">
-        <v>1</v>
-      </c>
-      <c r="D3" s="2">
+      <c r="A3" s="14">
+        <v>2</v>
+      </c>
+      <c r="B3" s="14">
+        <v>2</v>
+      </c>
+      <c r="C3" s="14">
+        <v>1</v>
+      </c>
+      <c r="D3" s="14">
         <v>14</v>
       </c>
-      <c r="E3" s="2">
-        <v>1</v>
-      </c>
-      <c r="F3" s="2">
-        <v>2</v>
-      </c>
-      <c r="G3" s="2">
+      <c r="E3" s="14">
+        <v>1</v>
+      </c>
+      <c r="F3" s="16">
+        <v>2</v>
+      </c>
+      <c r="G3" s="16">
         <v>2</v>
       </c>
     </row>

</xml_diff>